<commit_message>
Code entering in git , ready for next phase.
</commit_message>
<xml_diff>
--- a/POC_codebase.xlsx
+++ b/POC_codebase.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RAG_11\cursor ai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D109EC-5D90-4AB3-AF62-516ACE89DEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B482E696-79C2-4387-9940-07FB6017C608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A993DE83-7971-43AD-8B31-D4723355BAC9}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A993DE83-7971-43AD-8B31-D4723355BAC9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="codebase" sheetId="1" r:id="rId1"/>
+    <sheet name="Modules" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="597">
   <si>
     <t>SWC FEB</t>
   </si>
@@ -1538,13 +1539,1157 @@
   </si>
   <si>
     <t>FOLDER_STRUCT</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Total folders</t>
+  </si>
+  <si>
+    <t>OEM SWCs</t>
+  </si>
+  <si>
+    <t>Supplier SWCs</t>
+  </si>
+  <si>
+    <r>
+      <t>.c</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> files</t>
+    </r>
+  </si>
+  <si>
+    <t>20–22</t>
+  </si>
+  <si>
+    <r>
+      <t>.h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> files</t>
+    </r>
+  </si>
+  <si>
+    <t>Total source files</t>
+  </si>
+  <si>
+    <t>40–44</t>
+  </si>
+  <si>
+    <t>Functions</t>
+  </si>
+  <si>
+    <t>140–180</t>
+  </si>
+  <si>
+    <t>Global variables</t>
+  </si>
+  <si>
+    <t>40–60</t>
+  </si>
+  <si>
+    <r>
+      <t>Structures (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>struct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>25–35</t>
+  </si>
+  <si>
+    <t>Enums</t>
+  </si>
+  <si>
+    <t>20–30</t>
+  </si>
+  <si>
+    <t>Macros</t>
+  </si>
+  <si>
+    <t>80–120</t>
+  </si>
+  <si>
+    <t>Configuration constants</t>
+  </si>
+  <si>
+    <t>Calibration parameters</t>
+  </si>
+  <si>
+    <t>25–40</t>
+  </si>
+  <si>
+    <t>RTE APIs</t>
+  </si>
+  <si>
+    <t>30–50</t>
+  </si>
+  <si>
+    <t>CAN signals</t>
+  </si>
+  <si>
+    <t>Vehicle Status signals</t>
+  </si>
+  <si>
+    <t>35–50</t>
+  </si>
+  <si>
+    <t>Local variables</t>
+  </si>
+  <si>
+    <t>500–700</t>
+  </si>
+  <si>
+    <t>Function calls</t>
+  </si>
+  <si>
+    <t>500+</t>
+  </si>
+  <si>
+    <t>Include relationships</t>
+  </si>
+  <si>
+    <t>120–180</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Total C code</t>
+  </si>
+  <si>
+    <t>6,000–8,000 LOC</t>
+  </si>
+  <si>
+    <t>Executable C code</t>
+  </si>
+  <si>
+    <t>4,000–5,500 LOC</t>
+  </si>
+  <si>
+    <t>Header code</t>
+  </si>
+  <si>
+    <t>1,500–2,000 LOC</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>800–1,200 LOC</t>
+  </si>
+  <si>
+    <t>Total project size</t>
+  </si>
+  <si>
+    <t>7,000–9,000 LOC</t>
+  </si>
+  <si>
+    <t>CODE-BASE size</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">You now have your </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>foundation module</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, consisting of:</t>
+    </r>
+  </si>
+  <si>
+    <t>Common/</t>
+  </si>
+  <si>
+    <t>│</t>
+  </si>
+  <si>
+    <t>├── types.h</t>
+  </si>
+  <si>
+    <t>├── macros.h</t>
+  </si>
+  <si>
+    <t>├── constants.h</t>
+  </si>
+  <si>
+    <t>├── common.h</t>
+  </si>
+  <si>
+    <t>└── common.c</t>
+  </si>
+  <si>
+    <t>This module provides:</t>
+  </si>
+  <si>
+    <r>
+      <t>Shared data types (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>struct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>enum</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>typedef</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>Generic utility macros</t>
+  </si>
+  <si>
+    <t>Project-wide constants</t>
+  </si>
+  <si>
+    <t>Mathematical helper functions</t>
+  </si>
+  <si>
+    <t>Validation utilities</t>
+  </si>
+  <si>
+    <t>Object reset and copy functions</t>
+  </si>
+  <si>
+    <t>Timeout handling</t>
+  </si>
+  <si>
+    <t>Logging helpers</t>
+  </si>
+  <si>
+    <t>Every remaining SWC in the repository will depend on this module, making it the base layer for the ADAS project.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common Module </t>
+  </si>
+  <si>
+    <t>Configuration/</t>
+  </si>
+  <si>
+    <t>├── config.h</t>
+  </si>
+  <si>
+    <t>├── config.c</t>
+  </si>
+  <si>
+    <t>├── calibration.h</t>
+  </si>
+  <si>
+    <t>├── calibration.c</t>
+  </si>
+  <si>
+    <t>├── feature_config.h</t>
+  </si>
+  <si>
+    <t>├── feature_config.c</t>
+  </si>
+  <si>
+    <t>├── vehicle_variant.h</t>
+  </si>
+  <si>
+    <t>└── vehicle_variant.c</t>
+  </si>
+  <si>
+    <t>Purpose of Each Component</t>
+  </si>
+  <si>
+    <r>
+      <t>config</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Global software configuration (versions, diagnostics, logging, simulation mode).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>calibration</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Runtime tuning parameters such as TTC thresholds, speed limits, and collision probability thresholds.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>feature_config</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Enables or disables ADAS features without changing business logic.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>vehicle_variant</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Encapsulates region- and vehicle-specific behavior, allowing different variants (e.g., Sedan, SUV, Truck) and markets (EU, US, APAC).</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration Module </t>
+  </si>
+  <si>
+    <t>CANIF Module</t>
+  </si>
+  <si>
+    <t>CANIF/</t>
+  </si>
+  <si>
+    <t>├── can_if.h</t>
+  </si>
+  <si>
+    <t>├── can_if.c</t>
+  </si>
+  <si>
+    <t>├── can_parser.h</t>
+  </si>
+  <si>
+    <t>└── can_parser.c</t>
+  </si>
+  <si>
+    <r>
+      <t>can_if</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Provides the interface between the CAN driver and the ADAS software. Receives CAN frames, validates them, manages the RX queue, and dispatches frames to the parser.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>can_parser</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Decodes raw CAN frames into engineering values (vehicle speed, steering angle, brake status, gear position, etc.) and forwards the decoded signals to the Vehicle Status module.</t>
+    </r>
+  </si>
+  <si>
+    <t>Module Responsibilities</t>
+  </si>
+  <si>
+    <t>Receive CAN frames</t>
+  </si>
+  <si>
+    <t>Validate incoming frames</t>
+  </si>
+  <si>
+    <t>Maintain receive queue</t>
+  </si>
+  <si>
+    <t>Decode CAN messages</t>
+  </si>
+  <si>
+    <t>Convert raw bytes into physical values</t>
+  </si>
+  <si>
+    <t>Maintain parser statistics</t>
+  </si>
+  <si>
+    <t>Forward decoded vehicle signals to VehStatus</t>
+  </si>
+  <si>
+    <t>VehStatus Module</t>
+  </si>
+  <si>
+    <t>VehStatus/</t>
+  </si>
+  <si>
+    <t>├── vehstatus_in.h</t>
+  </si>
+  <si>
+    <t>├── vehstatus_in.c</t>
+  </si>
+  <si>
+    <t>├── vehstatus_out.h</t>
+  </si>
+  <si>
+    <t>└── vehstatus_out.c</t>
+  </si>
+  <si>
+    <r>
+      <t>vehstatus_in</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Receives decoded vehicle signals from the CAN Parser, validates them, updates the centralized vehicle status database, and maintains signal freshness.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>vehstatus_out</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Provides a read-only interface for all ADAS software components to access the latest vehicle status information without directly modifying the database.</t>
+    </r>
+  </si>
+  <si>
+    <t>Receive decoded CAN signals</t>
+  </si>
+  <si>
+    <t>Maintain centralized vehicle status database</t>
+  </si>
+  <si>
+    <t>Update vehicle motion state</t>
+  </si>
+  <si>
+    <t>Validate received vehicle data</t>
+  </si>
+  <si>
+    <t>Maintain update counters and timestamps</t>
+  </si>
+  <si>
+    <t>Provide read-only APIs for other modules</t>
+  </si>
+  <si>
+    <t>Act as the bridge between CANIF and RTE</t>
+  </si>
+  <si>
+    <t>RTE Module</t>
+  </si>
+  <si>
+    <t>RTE/</t>
+  </si>
+  <si>
+    <t>├── rte.h</t>
+  </si>
+  <si>
+    <t>├── rte.c</t>
+  </si>
+  <si>
+    <t>├── rte_read.h</t>
+  </si>
+  <si>
+    <t>├── rte_read.c</t>
+  </si>
+  <si>
+    <t>├── rte_write.h</t>
+  </si>
+  <si>
+    <t>└── rte_write.c</t>
+  </si>
+  <si>
+    <t>rte.h</t>
+  </si>
+  <si>
+    <t>Defines the core Runtime Environment interfaces and shared APIs for inter-module communication.</t>
+  </si>
+  <si>
+    <t>rte.c</t>
+  </si>
+  <si>
+    <t>Maintains the central ADAS runtime context and implements the core read/write services.</t>
+  </si>
+  <si>
+    <t>rte_read.h</t>
+  </si>
+  <si>
+    <t>Declares all read APIs used by application modules.</t>
+  </si>
+  <si>
+    <t>rte_read.c</t>
+  </si>
+  <si>
+    <t>Provides wrapper APIs for safely reading vehicle status, calibration, feature configuration, and FEB output.</t>
+  </si>
+  <si>
+    <t>rte_write.h</t>
+  </si>
+  <si>
+    <t>Declares write APIs for application modules.</t>
+  </si>
+  <si>
+    <t>rte_write.c</t>
+  </si>
+  <si>
+    <t>Implements wrapper APIs for updating runtime data.</t>
+  </si>
+  <si>
+    <t>Central communication layer between SWCs</t>
+  </si>
+  <si>
+    <t>Hide internal data structures from applications</t>
+  </si>
+  <si>
+    <t>Provide standardized Read/Write interfaces</t>
+  </si>
+  <si>
+    <t>Store current ADAS runtime context</t>
+  </si>
+  <si>
+    <t>Transfer vehicle status to all application components</t>
+  </si>
+  <si>
+    <t>Provide calibration and configuration access</t>
+  </si>
+  <si>
+    <t>Distribute FEB outputs to HMI and Display Manager</t>
+  </si>
+  <si>
+    <t>SWCCAM Module</t>
+  </si>
+  <si>
+    <t>SWCCAM/</t>
+  </si>
+  <si>
+    <t>├── camera_if.h</t>
+  </si>
+  <si>
+    <t>├── camera_if.c</t>
+  </si>
+  <si>
+    <t>├── camera_processing.h</t>
+  </si>
+  <si>
+    <t>├── camera_processing.c</t>
+  </si>
+  <si>
+    <t>├── lane_detection.h</t>
+  </si>
+  <si>
+    <t>├── lane_detection.c</t>
+  </si>
+  <si>
+    <t>├── object_detection.h</t>
+  </si>
+  <si>
+    <t>├── object_detection.c</t>
+  </si>
+  <si>
+    <t>├── camera_output.h</t>
+  </si>
+  <si>
+    <t>└── camera_output.c</t>
+  </si>
+  <si>
+    <t>camera_if</t>
+  </si>
+  <si>
+    <t>Interfaces with the camera sensor, receives raw camera frames, validates them, and stores the latest frame.</t>
+  </si>
+  <si>
+    <t>camera_processing</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Processes raw camera frames into standardized </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CameraObjectType</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> objects with confidence and signal quality.</t>
+    </r>
+  </si>
+  <si>
+    <t>lane_detection</t>
+  </si>
+  <si>
+    <t>Analyzes processed camera data to detect lane boundaries and generate lane information.</t>
+  </si>
+  <si>
+    <t>object_detection</t>
+  </si>
+  <si>
+    <t>Classifies detected camera objects (vehicle, pedestrian, cyclist, etc.) and prepares them for sensor fusion.</t>
+  </si>
+  <si>
+    <t>camera_output</t>
+  </si>
+  <si>
+    <t>Aggregates object detection and lane detection results into a single output package for downstream ADAS modules.</t>
+  </si>
+  <si>
+    <t>Acquire raw camera sensor frames.</t>
+  </si>
+  <si>
+    <t>Validate incoming camera data.</t>
+  </si>
+  <si>
+    <t>Process raw detections into camera objects.</t>
+  </si>
+  <si>
+    <t>Estimate lane information.</t>
+  </si>
+  <si>
+    <t>Detect and classify objects.</t>
+  </si>
+  <si>
+    <t>Assign confidence and signal quality.</t>
+  </si>
+  <si>
+    <t>Aggregate camera perception results.</t>
+  </si>
+  <si>
+    <t>Provide processed camera output to the Fusion module.</t>
+  </si>
+  <si>
+    <t>Serve as the perception layer for camera-based ADAS functions.</t>
+  </si>
+  <si>
+    <t>SWCRAD Module</t>
+  </si>
+  <si>
+    <t>SWCRAD/</t>
+  </si>
+  <si>
+    <t>├── swc_radar.h</t>
+  </si>
+  <si>
+    <t>├── swc_radar.c</t>
+  </si>
+  <si>
+    <t>├── radar_validation.h</t>
+  </si>
+  <si>
+    <t>└── radar_validation.c</t>
+  </si>
+  <si>
+    <t>swc_radar</t>
+  </si>
+  <si>
+    <t>Receives validated radar detections, manages radar processing, and publishes processed radar objects for the Sensor Fusion module.</t>
+  </si>
+  <si>
+    <t>radar_validation</t>
+  </si>
+  <si>
+    <t>Validates raw radar detections by checking measurement limits, filtering invalid targets, assigning signal quality, and providing validated radar objects to the Radar SWC.</t>
+  </si>
+  <si>
+    <t>Acquire radar detections.</t>
+  </si>
+  <si>
+    <t>Validate radar measurements.</t>
+  </si>
+  <si>
+    <t>Filter invalid radar targets.</t>
+  </si>
+  <si>
+    <t>Assign signal quality to radar objects.</t>
+  </si>
+  <si>
+    <t>Maintain processed radar object list.</t>
+  </si>
+  <si>
+    <t>Provide radar objects to the Fusion module.</t>
+  </si>
+  <si>
+    <t>Support downstream collision detection and object fusion.</t>
+  </si>
+  <si>
+    <t>Act as the radar perception layer within the ADAS pipeline.</t>
+  </si>
+  <si>
+    <t>SWCFUSION Module</t>
+  </si>
+  <si>
+    <t>SWCFUSION/</t>
+  </si>
+  <si>
+    <t>├── swc_fusion.h</t>
+  </si>
+  <si>
+    <t>├── swc_fusion.c</t>
+  </si>
+  <si>
+    <t>├── fusion_filter.h</t>
+  </si>
+  <si>
+    <t>└── fusion_filter.c</t>
+  </si>
+  <si>
+    <t>swc_fusion</t>
+  </si>
+  <si>
+    <t>Coordinates the sensor fusion workflow by collecting processed camera and radar data, invoking the fusion algorithm, and publishing fused objects for downstream ADAS modules.</t>
+  </si>
+  <si>
+    <t>fusion_filter</t>
+  </si>
+  <si>
+    <t>Associates camera and radar detections, computes fused object attributes such as distance, relative speed, time-to-collision (TTC), and collision probability, and generates the unified object list consumed by the FEB module.</t>
+  </si>
+  <si>
+    <t>Receive processed camera perception data.</t>
+  </si>
+  <si>
+    <t>Receive validated radar detections.</t>
+  </si>
+  <si>
+    <t>Associate camera and radar objects.</t>
+  </si>
+  <si>
+    <t>Generate fused object list.</t>
+  </si>
+  <si>
+    <t>Calculate distance to target.</t>
+  </si>
+  <si>
+    <t>Calculate relative speed.</t>
+  </si>
+  <si>
+    <t>Calculate Time-To-Collision (TTC).</t>
+  </si>
+  <si>
+    <t>Estimate collision probability.</t>
+  </si>
+  <si>
+    <t>Validate fused objects.</t>
+  </si>
+  <si>
+    <t>Publish fusion output to the FEB software component.</t>
+  </si>
+  <si>
+    <t>SWCFEB Module</t>
+  </si>
+  <si>
+    <t>SWCFEB/</t>
+  </si>
+  <si>
+    <t>├── swc_feb.h</t>
+  </si>
+  <si>
+    <t>├── swc_feb.c</t>
+  </si>
+  <si>
+    <t>├── feb_logic.h</t>
+  </si>
+  <si>
+    <t>├── feb_logic.c</t>
+  </si>
+  <si>
+    <t>├── feb_output.h</t>
+  </si>
+  <si>
+    <t>└── feb_output.c</t>
+  </si>
+  <si>
+    <t>swc_feb</t>
+  </si>
+  <si>
+    <t>Coordinates the complete Forward Emergency Braking pipeline by receiving fused objects, invoking the braking decision logic, and publishing the final FEB output.</t>
+  </si>
+  <si>
+    <t>feb_logic</t>
+  </si>
+  <si>
+    <t>Implements the Forward Emergency Braking decision algorithm by evaluating fused objects against calibration parameters to determine warning and brake requests.</t>
+  </si>
+  <si>
+    <t>feb_output</t>
+  </si>
+  <si>
+    <t>Stores, validates, and provides the latest FEB output to downstream modules such as HMI, Display Manager, Diagnostics, and supplier software.</t>
+  </si>
+  <si>
+    <t>Receive fused perception objects.</t>
+  </si>
+  <si>
+    <t>Identify the most critical collision target.</t>
+  </si>
+  <si>
+    <t>Calculate braking decisions using TTC thresholds.</t>
+  </si>
+  <si>
+    <t>Generate driver warning requests.</t>
+  </si>
+  <si>
+    <t>Generate automatic brake requests.</t>
+  </si>
+  <si>
+    <t>Maintain FEB system state.</t>
+  </si>
+  <si>
+    <t>Publish FEB outputs.</t>
+  </si>
+  <si>
+    <t>Provide braking information to HMI, Display Manager, Diagnostics, and Supplier FEB.</t>
+  </si>
+  <si>
+    <t>SWCHMI Module</t>
+  </si>
+  <si>
+    <t>SWCHMI/</t>
+  </si>
+  <si>
+    <t>├── swc_hmi.h</t>
+  </si>
+  <si>
+    <t>└── swc_hmi.c</t>
+  </si>
+  <si>
+    <t>swc_hmi</t>
+  </si>
+  <si>
+    <t>Receives the Forward Emergency Braking output and converts it into driver-facing indications such as visual warnings, audible alerts, and display messages for the Display Manager.</t>
+  </si>
+  <si>
+    <t>Receive FEB output.</t>
+  </si>
+  <si>
+    <t>Generate driver warning indications.</t>
+  </si>
+  <si>
+    <t>Control warning lamp status.</t>
+  </si>
+  <si>
+    <t>Control audible buzzer activation.</t>
+  </si>
+  <si>
+    <t>Generate display message requests.</t>
+  </si>
+  <si>
+    <t>Provide processed HMI output to the Display Manager.</t>
+  </si>
+  <si>
+    <t>DisplayManager Module</t>
+  </si>
+  <si>
+    <t>DisplayManager/</t>
+  </si>
+  <si>
+    <t>├── display_manager.h</t>
+  </si>
+  <si>
+    <t>└── display_manager.c</t>
+  </si>
+  <si>
+    <t>display_manager</t>
+  </si>
+  <si>
+    <t>Receives processed HMI information and converts it into dashboard display requests such as warning icons, brake icons, text messages, and buzzer requests for the vehicle's instrument cluster or HUD.</t>
+  </si>
+  <si>
+    <t>Receive processed HMI output.</t>
+  </si>
+  <si>
+    <t>Generate dashboard warning indications.</t>
+  </si>
+  <si>
+    <t>Control warning icon display.</t>
+  </si>
+  <si>
+    <t>Control brake icon display.</t>
+  </si>
+  <si>
+    <t>Generate driver text messages.</t>
+  </si>
+  <si>
+    <t>Forward buzzer requests.</t>
+  </si>
+  <si>
+    <t>Provide finalized display information to the vehicle display system.</t>
+  </si>
+  <si>
+    <t>Diagnostics Module</t>
+  </si>
+  <si>
+    <t>Diagnostics/</t>
+  </si>
+  <si>
+    <t>├── diagnostics.h</t>
+  </si>
+  <si>
+    <t>└── diagnostics.c</t>
+  </si>
+  <si>
+    <t>diagnostics</t>
+  </si>
+  <si>
+    <t>Monitors the health and operational state of ADAS software components, maintains diagnostic records, detects communication failures, and provides diagnostic information for debugging and service tools.</t>
+  </si>
+  <si>
+    <t>Monitor software component health.</t>
+  </si>
+  <si>
+    <t>Track module operational states.</t>
+  </si>
+  <si>
+    <t>Record communication failures.</t>
+  </si>
+  <si>
+    <t>Maintain diagnostic records.</t>
+  </si>
+  <si>
+    <t>Count runtime errors.</t>
+  </si>
+  <si>
+    <t>Provide diagnostic information for service and debugging.</t>
+  </si>
+  <si>
+    <t>Support overall ADAS system health monitoring.</t>
+  </si>
+  <si>
+    <t>Application Module</t>
+  </si>
+  <si>
+    <t>Application/</t>
+  </si>
+  <si>
+    <t>├── scheduler.h</t>
+  </si>
+  <si>
+    <t>├── scheduler.c</t>
+  </si>
+  <si>
+    <t>└── main.c</t>
+  </si>
+  <si>
+    <t>scheduler</t>
+  </si>
+  <si>
+    <t>Initializes all ADAS software components and executes them in the required cyclic order, ensuring correct data flow across the entire ADAS pipeline.</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>Entry point of the ADAS application. Initializes the scheduler and continuously executes the ADAS processing loop.</t>
+  </si>
+  <si>
+    <t>Initialize the complete ADAS software stack.</t>
+  </si>
+  <si>
+    <t>Execute software components in the correct sequence.</t>
+  </si>
+  <si>
+    <t>Coordinate data flow between modules.</t>
+  </si>
+  <si>
+    <t>Maintain the cyclic execution of the ADAS application.</t>
+  </si>
+  <si>
+    <t>Serve as the top-level control of the entire ADAS system.</t>
+  </si>
+  <si>
+    <t>SUPSWC/SWCFEB_SUP Module</t>
+  </si>
+  <si>
+    <t>SUPSWC/</t>
+  </si>
+  <si>
+    <t>└── SWCFEB_SUP/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ├── supplier_feb.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    └── supplier_feb.c</t>
+  </si>
+  <si>
+    <t>supplier_feb</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Represents a third-party supplier implementation of the Forward Emergency Braking (FEB) algorithm. It provides an OEM-independent interface that processes fused object data using calibration parameters and generates braking and warning requests. The OEM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SWCFEB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> module can invoke this interface instead of embedding supplier-specific logic directly.</t>
+    </r>
+  </si>
+  <si>
+    <t>Simulate a supplier-owned FEB component.</t>
+  </si>
+  <si>
+    <t>Process fused object information.</t>
+  </si>
+  <si>
+    <t>Retrieve FEB calibration values.</t>
+  </si>
+  <si>
+    <t>Evaluate Time-To-Collision (TTC).</t>
+  </si>
+  <si>
+    <t>Generate warning and brake requests.</t>
+  </si>
+  <si>
+    <t>Return standardized FEB outputs.</t>
+  </si>
+  <si>
+    <t>Maintain OEM–Supplier architectural separation.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1589,8 +2734,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1600,6 +2753,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1668,7 +2827,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1730,6 +2889,33 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1739,32 +2925,32 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1850,8 +3036,8 @@
     <xdr:to>
       <xdr:col>20</xdr:col>
       <xdr:colOff>1607799</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>39951</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>27394</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1894,8 +3080,8 @@
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>107028</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>227420</xdr:rowOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>36920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2393,37 +3579,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF7F3584-E6E4-49A1-8CAA-8668E54A8948}">
   <dimension ref="B2:U214"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9.06640625" style="4"/>
-    <col min="2" max="2" width="38.73046875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="9.06640625" style="4"/>
+    <col min="2" max="2" width="37.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.06640625" style="4"/>
+    <col min="4" max="4" width="50.19921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.06640625" style="4"/>
+    <col min="6" max="6" width="71.1328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.06640625" style="4"/>
     <col min="8" max="8" width="25" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.06640625" style="4"/>
     <col min="10" max="10" width="29.6640625" style="4" customWidth="1"/>
     <col min="11" max="11" width="9.06640625" style="4"/>
     <col min="12" max="12" width="23.1328125" style="4" customWidth="1"/>
-    <col min="13" max="13" width="9.9296875" style="4" customWidth="1"/>
-    <col min="14" max="14" width="39.1328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.9296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="37.73046875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="63.53125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="74.06640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.06640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.86328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="38.59765625" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="52.86328125" style="4" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="29" style="4" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.06640625" style="4" customWidth="1"/>
     <col min="21" max="21" width="23.53125" style="4" bestFit="1" customWidth="1"/>
     <col min="22" max="16384" width="9.06640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:21">
       <c r="B2" s="3"/>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
       <c r="N2" s="3" t="s">
         <v>7</v>
       </c>
@@ -2434,202 +3624,202 @@
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
     </row>
-    <row r="3" spans="2:21" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:21">
       <c r="B3" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="T3" s="21" t="s">
+      <c r="T3" s="30" t="s">
         <v>301</v>
       </c>
-      <c r="U3" s="21"/>
-    </row>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="U3" s="30"/>
+    </row>
+    <row r="4" spans="2:21">
       <c r="B4" s="4" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="5" spans="2:21" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:21">
       <c r="B5" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="H5" s="27" t="s">
+      <c r="H5" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="L5" s="27" t="s">
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="L5" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="M5" s="27"/>
-    </row>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="M5" s="28"/>
+    </row>
+    <row r="6" spans="2:21">
       <c r="B6" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-    </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+    </row>
+    <row r="7" spans="2:21">
       <c r="B7" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="H7" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
-      <c r="O7" s="27" t="s">
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="O7" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
-    </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+    </row>
+    <row r="8" spans="2:21">
       <c r="B8" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="O8" s="27"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="27"/>
-    </row>
-    <row r="9" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="28"/>
+    </row>
+    <row r="9" spans="2:21">
       <c r="B9" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="H9" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="L9" s="27" t="s">
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="L9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="M9" s="27"/>
-      <c r="O9" s="28" t="s">
+      <c r="M9" s="28"/>
+      <c r="O9" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="28"/>
-    </row>
-    <row r="10" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
+    </row>
+    <row r="10" spans="2:21">
       <c r="B10" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="L10" s="27"/>
-      <c r="M10" s="27"/>
-      <c r="O10" s="28"/>
-      <c r="P10" s="28"/>
-      <c r="Q10" s="28"/>
-    </row>
-    <row r="11" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="O10" s="29"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="29"/>
+    </row>
+    <row r="11" spans="2:21">
       <c r="B11" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
-      <c r="O11" s="28"/>
-      <c r="P11" s="28"/>
-      <c r="Q11" s="28"/>
-    </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="O11" s="29"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
+    </row>
+    <row r="12" spans="2:21">
       <c r="B12" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="O12" s="28"/>
-      <c r="P12" s="28"/>
-      <c r="Q12" s="28"/>
-    </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
+      <c r="O12" s="29"/>
+      <c r="P12" s="29"/>
+      <c r="Q12" s="29"/>
+    </row>
+    <row r="13" spans="2:21">
       <c r="B13" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-      <c r="L13" s="27" t="s">
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
+      <c r="L13" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="M13" s="27"/>
-      <c r="O13" s="28"/>
-      <c r="P13" s="28"/>
-      <c r="Q13" s="28"/>
-    </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="M13" s="28"/>
+      <c r="O13" s="29"/>
+      <c r="P13" s="29"/>
+      <c r="Q13" s="29"/>
+    </row>
+    <row r="14" spans="2:21">
       <c r="B14" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="27"/>
-      <c r="O14" s="28"/>
-      <c r="P14" s="28"/>
-      <c r="Q14" s="28"/>
-    </row>
-    <row r="15" spans="2:21" x14ac:dyDescent="0.45">
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="O14" s="29"/>
+      <c r="P14" s="29"/>
+      <c r="Q14" s="29"/>
+    </row>
+    <row r="15" spans="2:21">
       <c r="B15" s="4" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="16" spans="2:21" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:21">
       <c r="B16" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="H16" s="27" t="s">
+      <c r="H16" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-    </row>
-    <row r="17" spans="2:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28"/>
+    </row>
+    <row r="17" spans="2:18">
       <c r="B17" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="H17" s="28" t="s">
+      <c r="H17" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="28"/>
-    </row>
-    <row r="18" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="I17" s="29"/>
+      <c r="J17" s="29"/>
+      <c r="K17" s="29"/>
+    </row>
+    <row r="18" spans="2:18">
       <c r="B18" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="28"/>
-    </row>
-    <row r="19" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="H18" s="29"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="29"/>
+      <c r="K18" s="29"/>
+    </row>
+    <row r="19" spans="2:18">
       <c r="B19" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
-    </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="29"/>
+    </row>
+    <row r="20" spans="2:18">
       <c r="B20" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
       <c r="M20" s="15" t="s">
         <v>185</v>
       </c>
@@ -2642,20 +3832,20 @@
       <c r="P20" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="Q20" s="30" t="s">
+      <c r="Q20" s="33" t="s">
         <v>300</v>
       </c>
-      <c r="R20" s="31"/>
-    </row>
-    <row r="21" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="R20" s="34"/>
+    </row>
+    <row r="21" spans="2:18" ht="28.5">
       <c r="B21" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="H21" s="28"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="M21" s="32" t="s">
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
+      <c r="M21" s="22" t="s">
         <v>290</v>
       </c>
       <c r="N21" s="10" t="s">
@@ -2664,21 +3854,21 @@
       <c r="O21" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="P21" s="29" t="s">
+      <c r="P21" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="Q21" s="31"/>
-      <c r="R21" s="31"/>
-    </row>
-    <row r="22" spans="2:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="Q21" s="34"/>
+      <c r="R21" s="34"/>
+    </row>
+    <row r="22" spans="2:18" ht="28.5">
       <c r="B22" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="28"/>
-      <c r="M22" s="32" t="s">
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="M22" s="22" t="s">
         <v>293</v>
       </c>
       <c r="N22" s="10" t="s">
@@ -2687,21 +3877,21 @@
       <c r="O22" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="P22" s="29" t="s">
+      <c r="P22" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="Q22" s="31"/>
-      <c r="R22" s="31"/>
-    </row>
-    <row r="23" spans="2:18" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="Q22" s="34"/>
+      <c r="R22" s="34"/>
+    </row>
+    <row r="23" spans="2:18" ht="42.75">
       <c r="B23" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
-      <c r="M23" s="32" t="s">
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="M23" s="22" t="s">
         <v>297</v>
       </c>
       <c r="N23" s="10" t="s">
@@ -2710,25 +3900,75 @@
       <c r="O23" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="P23" s="29" t="s">
+      <c r="P23" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
-    </row>
-    <row r="24" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="Q23" s="34"/>
+      <c r="R23" s="34"/>
+    </row>
+    <row r="24" spans="2:18">
       <c r="B24" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
-    </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="Q24" s="34"/>
+      <c r="R24" s="34"/>
+    </row>
+    <row r="25" spans="2:18">
       <c r="B25" s="4" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="33" spans="3:10" ht="23.25" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:18">
+      <c r="L29" s="26" t="s">
+        <v>347</v>
+      </c>
+      <c r="M29" s="26"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
+    </row>
+    <row r="30" spans="2:18">
+      <c r="L30" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="M30" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="N30" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="O30" s="23" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="31" spans="2:18">
+      <c r="L31" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="M31" s="23">
+        <v>14</v>
+      </c>
+      <c r="N31" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="O31" s="23" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="32" spans="2:18">
+      <c r="L32" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="M32" s="23">
+        <v>13</v>
+      </c>
+      <c r="N32" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="O32" s="23" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="33" spans="3:15" ht="23.25">
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
         <v>30</v>
@@ -2739,143 +3979,277 @@
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
-    </row>
-    <row r="35" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L33" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="M33" s="23">
+        <v>1</v>
+      </c>
+      <c r="N33" s="10" t="s">
+        <v>341</v>
+      </c>
+      <c r="O33" s="23" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="34" spans="3:15">
+      <c r="L34" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="M34" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="N34" s="10" t="s">
+        <v>343</v>
+      </c>
+      <c r="O34" s="23" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="35" spans="3:15">
       <c r="F35" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="37" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L35" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="M35" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="N35" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="O35" s="23" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="36" spans="3:15">
+      <c r="L36" s="9" t="s">
+        <v>310</v>
+      </c>
+      <c r="M36" s="23" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="37" spans="3:15">
       <c r="F37" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="39" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L37" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="M37" s="23" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="38" spans="3:15">
+      <c r="L38" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="M38" s="23" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="39" spans="3:15">
       <c r="F39" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="41" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L39" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="M39" s="23" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="40" spans="3:15">
+      <c r="L40" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="M40" s="23" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="41" spans="3:15">
       <c r="F41" s="11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="43" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L41" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="M41" s="23" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="42" spans="3:15">
+      <c r="L42" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="M42" s="23" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="43" spans="3:15">
       <c r="F43" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="44" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L43" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="M43" s="23" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="44" spans="3:15">
       <c r="F44" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="45" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L44" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="M44" s="23" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="45" spans="3:15">
       <c r="F45" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="47" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="L45" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="M45" s="23" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="46" spans="3:15">
+      <c r="L46" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="M46" s="23" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="47" spans="3:15">
       <c r="F47" s="11" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.45">
+      <c r="L47" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="M47" s="23" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="48" spans="3:15">
+      <c r="L48" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="M48" s="23" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="49" spans="6:13">
       <c r="F49" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.45">
+      <c r="L49" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="M49" s="23" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="50" spans="6:13">
       <c r="F50" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="51" spans="6:13">
       <c r="F51" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="52" spans="6:13">
       <c r="F52" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="53" spans="6:13">
       <c r="F53" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="55" spans="6:13">
       <c r="F55" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="57" spans="6:13">
       <c r="F57" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="58" spans="6:13">
       <c r="F58" s="12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="59" spans="6:13">
       <c r="F59" s="12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="60" spans="6:13">
       <c r="F60" s="12" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="61" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="61" spans="6:13">
       <c r="F61" s="12" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="63" spans="6:13">
       <c r="F63" s="12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="6:6" x14ac:dyDescent="0.45">
+    <row r="64" spans="6:13">
       <c r="F64" s="12" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="65" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="65" spans="6:18">
       <c r="F65" s="12" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="66" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="66" spans="6:18">
       <c r="F66" s="12" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="67" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="67" spans="6:18">
       <c r="F67" s="12" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="69" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="69" spans="6:18">
       <c r="F69" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="73" spans="6:18" ht="23.25" x14ac:dyDescent="0.45">
+    <row r="73" spans="6:18" ht="23.25">
       <c r="F73" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="74" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="74" spans="6:18">
       <c r="L74" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="M74" s="25"/>
-      <c r="N74" s="26"/>
+      <c r="M74" s="27"/>
+      <c r="N74" s="25"/>
       <c r="P74" s="15" t="s">
         <v>185</v>
       </c>
@@ -2886,7 +4260,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="75" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="75" spans="6:18">
       <c r="F75" s="11" t="s">
         <v>57</v>
       </c>
@@ -2909,7 +4283,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="76" spans="6:18" ht="42.75">
       <c r="L76" s="9" t="s">
         <v>86</v>
       </c>
@@ -2929,7 +4303,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="77" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="77" spans="6:18" ht="42.75">
       <c r="F77" s="11" t="s">
         <v>32</v>
       </c>
@@ -2952,7 +4326,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="78" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="78" spans="6:18" ht="71.25">
       <c r="L78" s="9" t="s">
         <v>201</v>
       </c>
@@ -2964,7 +4338,7 @@
       </c>
       <c r="Q78" s="7"/>
     </row>
-    <row r="79" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="79" spans="6:18" ht="85.5">
       <c r="F79" s="4" t="s">
         <v>58</v>
       </c>
@@ -2980,9 +4354,9 @@
       <c r="Q79" s="24" t="s">
         <v>263</v>
       </c>
-      <c r="R79" s="26"/>
-    </row>
-    <row r="80" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+      <c r="R79" s="25"/>
+    </row>
+    <row r="80" spans="6:18" ht="27">
       <c r="F80" s="4" t="s">
         <v>59</v>
       </c>
@@ -3002,7 +4376,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="81" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="81" spans="6:18">
       <c r="L81" s="9" t="s">
         <v>210</v>
       </c>
@@ -3019,7 +4393,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="82" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="82" spans="6:18" ht="27">
       <c r="F82" s="11" t="s">
         <v>38</v>
       </c>
@@ -3039,7 +4413,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="83" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="83" spans="6:18" ht="39.75">
       <c r="L83" s="9" t="s">
         <v>90</v>
       </c>
@@ -3056,7 +4430,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="84" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="84" spans="6:18" ht="27">
       <c r="F84" s="4" t="s">
         <v>60</v>
       </c>
@@ -3076,7 +4450,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="85" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="85" spans="6:18" ht="27">
       <c r="F85" s="4" t="s">
         <v>61</v>
       </c>
@@ -3096,7 +4470,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="86" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="86" spans="6:18">
       <c r="F86" s="4" t="s">
         <v>62</v>
       </c>
@@ -3113,7 +4487,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="87" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="87" spans="6:18" ht="27">
       <c r="F87" s="4" t="s">
         <v>63</v>
       </c>
@@ -3130,7 +4504,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="88" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="88" spans="6:18" ht="27">
       <c r="F88" s="4" t="s">
         <v>64</v>
       </c>
@@ -3147,7 +4521,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="89" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="89" spans="6:18" ht="27">
       <c r="F89" s="4" t="s">
         <v>65</v>
       </c>
@@ -3164,7 +4538,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="90" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="90" spans="6:18" ht="27">
       <c r="L90" s="9" t="s">
         <v>229</v>
       </c>
@@ -3178,7 +4552,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="91" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="91" spans="6:18">
       <c r="F91" s="4" t="s">
         <v>66</v>
       </c>
@@ -3195,7 +4569,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="92" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="92" spans="6:18" ht="27">
       <c r="L92" s="9" t="s">
         <v>99</v>
       </c>
@@ -3209,7 +4583,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="93" spans="6:18" ht="52.5" x14ac:dyDescent="0.45">
+    <row r="93" spans="6:18" ht="27">
       <c r="F93" s="12" t="s">
         <v>21</v>
       </c>
@@ -3226,7 +4600,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="94" spans="6:18" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="94" spans="6:18" ht="27">
       <c r="L94" s="9" t="s">
         <v>101</v>
       </c>
@@ -3240,7 +4614,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="95" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="95" spans="6:18">
       <c r="L95" s="14"/>
       <c r="M95" s="16"/>
       <c r="N95" s="7"/>
@@ -3248,7 +4622,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="96" spans="6:18" x14ac:dyDescent="0.45">
+    <row r="96" spans="6:18">
       <c r="L96" s="14"/>
       <c r="M96" s="16"/>
       <c r="N96" s="7"/>
@@ -3256,19 +4630,19 @@
         <v>251</v>
       </c>
     </row>
-    <row r="97" spans="6:17" x14ac:dyDescent="0.45">
+    <row r="97" spans="6:17">
       <c r="F97" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="L97" s="22" t="s">
+      <c r="L97" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="M97" s="23"/>
+      <c r="M97" s="32"/>
       <c r="Q97" s="20" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="98" spans="6:17" ht="17.649999999999999" x14ac:dyDescent="0.45">
+    <row r="98" spans="6:17" ht="17.649999999999999">
       <c r="L98" s="8" t="s">
         <v>103</v>
       </c>
@@ -3279,7 +4653,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="99" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="99" spans="6:17">
       <c r="F99" s="12" t="s">
         <v>68</v>
       </c>
@@ -3293,7 +4667,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="100" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="100" spans="6:17">
       <c r="L100" s="2">
         <v>2</v>
       </c>
@@ -3304,7 +4678,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="101" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="101" spans="6:17">
       <c r="F101" s="12" t="s">
         <v>16</v>
       </c>
@@ -3318,7 +4692,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="102" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="102" spans="6:17">
       <c r="L102" s="2">
         <v>4</v>
       </c>
@@ -3329,7 +4703,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="103" spans="6:17" x14ac:dyDescent="0.45">
+    <row r="103" spans="6:17">
       <c r="F103" s="12" t="s">
         <v>69</v>
       </c>
@@ -3343,7 +4717,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="104" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="104" spans="6:17">
       <c r="L104" s="2">
         <v>6</v>
       </c>
@@ -3354,7 +4728,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="105" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="105" spans="6:17" ht="17.649999999999999">
       <c r="F105" s="12" t="s">
         <v>27</v>
       </c>
@@ -3368,24 +4742,24 @@
         <v>98</v>
       </c>
     </row>
-    <row r="106" spans="6:17" x14ac:dyDescent="0.45">
+    <row r="106" spans="6:17">
       <c r="Q106" s="20" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="107" spans="6:17" x14ac:dyDescent="0.45">
+    <row r="107" spans="6:17">
       <c r="F107" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="L107" s="22" t="s">
+      <c r="L107" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="M107" s="23"/>
+      <c r="M107" s="32"/>
       <c r="Q107" s="20" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="108" spans="6:17" ht="57" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="108" spans="6:17">
       <c r="L108" s="8" t="s">
         <v>111</v>
       </c>
@@ -3396,7 +4770,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="109" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="109" spans="6:17">
       <c r="F109" s="12" t="s">
         <v>29</v>
       </c>
@@ -3410,7 +4784,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="110" spans="6:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="110" spans="6:17" ht="28.5">
       <c r="L110" s="2">
         <v>2</v>
       </c>
@@ -3418,7 +4792,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="111" spans="6:17" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="111" spans="6:17" ht="28.5">
       <c r="F111" s="12" t="s">
         <v>71</v>
       </c>
@@ -3429,7 +4803,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="112" spans="6:17" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="112" spans="6:17" ht="28.5">
       <c r="L112" s="2">
         <v>4</v>
       </c>
@@ -3437,7 +4811,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="113" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="113" spans="6:13" ht="28.5">
       <c r="F113" s="4" t="s">
         <v>72</v>
       </c>
@@ -3448,7 +4822,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="114" spans="6:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="114" spans="6:13" ht="28.5">
       <c r="L114" s="2">
         <v>6</v>
       </c>
@@ -3456,7 +4830,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="115" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="115" spans="6:13" ht="28.5">
       <c r="L115" s="2">
         <v>7</v>
       </c>
@@ -3464,7 +4838,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="116" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="116" spans="6:13" ht="28.5">
       <c r="L116" s="2">
         <v>8</v>
       </c>
@@ -3472,19 +4846,19 @@
         <v>118</v>
       </c>
     </row>
-    <row r="117" spans="6:13" ht="23.25" x14ac:dyDescent="0.45">
+    <row r="117" spans="6:13" ht="23.25">
       <c r="F117" s="6" t="s">
         <v>73</v>
       </c>
       <c r="L117" s="13"/>
     </row>
-    <row r="118" spans="6:13" x14ac:dyDescent="0.45">
-      <c r="L118" s="22" t="s">
+    <row r="118" spans="6:13">
+      <c r="L118" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="M118" s="23"/>
-    </row>
-    <row r="119" spans="6:13" x14ac:dyDescent="0.45">
+      <c r="M118" s="32"/>
+    </row>
+    <row r="119" spans="6:13">
       <c r="F119" s="11" t="s">
         <v>74</v>
       </c>
@@ -3495,7 +4869,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="120" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="120" spans="6:13" ht="28.5">
       <c r="L120" s="2">
         <v>1</v>
       </c>
@@ -3503,7 +4877,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="121" spans="6:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="121" spans="6:13" ht="28.5">
       <c r="F121" s="4" t="s">
         <v>75</v>
       </c>
@@ -3514,7 +4888,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="122" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="122" spans="6:13" ht="28.5">
       <c r="L122" s="2">
         <v>3</v>
       </c>
@@ -3522,7 +4896,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="123" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="123" spans="6:13" ht="28.5">
       <c r="F123" s="11" t="s">
         <v>32</v>
       </c>
@@ -3533,7 +4907,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="124" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="124" spans="6:13" ht="28.5">
       <c r="L124" s="2">
         <v>5</v>
       </c>
@@ -3541,23 +4915,23 @@
         <v>124</v>
       </c>
     </row>
-    <row r="125" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="125" spans="6:13">
       <c r="F125" s="4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="126" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="126" spans="6:13">
       <c r="F126" s="4" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="127" spans="6:13" x14ac:dyDescent="0.45">
-      <c r="L127" s="22" t="s">
+    <row r="127" spans="6:13">
+      <c r="L127" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="M127" s="23"/>
-    </row>
-    <row r="128" spans="6:13" x14ac:dyDescent="0.45">
+      <c r="M127" s="32"/>
+    </row>
+    <row r="128" spans="6:13">
       <c r="F128" s="11" t="s">
         <v>38</v>
       </c>
@@ -3568,7 +4942,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="129" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="129" spans="6:13">
       <c r="L129" s="2">
         <v>1</v>
       </c>
@@ -3576,7 +4950,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="130" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="130" spans="6:13">
       <c r="F130" s="4" t="s">
         <v>78</v>
       </c>
@@ -3587,7 +4961,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="131" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="131" spans="6:13" ht="28.5">
       <c r="F131" s="4" t="s">
         <v>79</v>
       </c>
@@ -3598,7 +4972,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="132" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="132" spans="6:13" ht="28.5">
       <c r="F132" s="4" t="s">
         <v>80</v>
       </c>
@@ -3609,7 +4983,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="133" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="133" spans="6:13" ht="28.5">
       <c r="F133" s="4" t="s">
         <v>81</v>
       </c>
@@ -3620,7 +4994,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="134" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="134" spans="6:13" ht="28.5">
       <c r="F134" s="4" t="s">
         <v>82</v>
       </c>
@@ -3631,7 +5005,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="135" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="135" spans="6:13" ht="28.5">
       <c r="L135" s="2">
         <v>7</v>
       </c>
@@ -3639,7 +5013,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="136" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="136" spans="6:13" ht="28.5">
       <c r="F136" s="4" t="s">
         <v>66</v>
       </c>
@@ -3650,21 +5024,21 @@
         <v>133</v>
       </c>
     </row>
-    <row r="138" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="138" spans="6:13">
       <c r="F138" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="139" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="139" spans="6:13">
       <c r="F139" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="L139" s="22" t="s">
+      <c r="L139" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="M139" s="23"/>
-    </row>
-    <row r="140" spans="6:13" x14ac:dyDescent="0.45">
+      <c r="M139" s="32"/>
+    </row>
+    <row r="140" spans="6:13">
       <c r="L140" s="1" t="s">
         <v>125</v>
       </c>
@@ -3672,7 +5046,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="141" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="141" spans="6:13" ht="28.5">
       <c r="F141" s="12" t="s">
         <v>21</v>
       </c>
@@ -3683,7 +5057,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="142" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="142" spans="6:13" ht="28.5">
       <c r="F142" s="12" t="s">
         <v>22</v>
       </c>
@@ -3694,7 +5068,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="143" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="143" spans="6:13" ht="28.5">
       <c r="L143" s="2">
         <v>3</v>
       </c>
@@ -3702,7 +5076,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="144" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="144" spans="6:13" ht="28.5">
       <c r="F144" s="12" t="s">
         <v>23</v>
       </c>
@@ -3713,7 +5087,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="145" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="145" spans="6:13" ht="28.5">
       <c r="L145" s="2">
         <v>5</v>
       </c>
@@ -3721,30 +5095,30 @@
         <v>138</v>
       </c>
     </row>
-    <row r="146" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="146" spans="6:13">
       <c r="F146" s="12" t="s">
         <v>12</v>
       </c>
       <c r="L146" s="13"/>
       <c r="M146" s="13"/>
     </row>
-    <row r="147" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="147" spans="6:13">
       <c r="F147" s="12" t="s">
         <v>24</v>
       </c>
       <c r="L147" s="13"/>
       <c r="M147" s="13"/>
     </row>
-    <row r="148" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="148" spans="6:13">
       <c r="F148" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="L148" s="22" t="s">
+      <c r="L148" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="M148" s="23"/>
-    </row>
-    <row r="149" spans="6:13" x14ac:dyDescent="0.45">
+      <c r="M148" s="32"/>
+    </row>
+    <row r="149" spans="6:13">
       <c r="F149" s="12" t="s">
         <v>24</v>
       </c>
@@ -3755,7 +5129,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="150" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="150" spans="6:13">
       <c r="F150" s="12" t="s">
         <v>14</v>
       </c>
@@ -3766,7 +5140,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="151" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="151" spans="6:13" ht="28.5">
       <c r="F151" s="12" t="s">
         <v>24</v>
       </c>
@@ -3777,7 +5151,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="152" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="152" spans="6:13" ht="28.5">
       <c r="F152" s="12" t="s">
         <v>18</v>
       </c>
@@ -3788,7 +5162,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="153" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="153" spans="6:13" ht="28.5">
       <c r="F153" s="12" t="s">
         <v>24</v>
       </c>
@@ -3799,7 +5173,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="154" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="154" spans="6:13" ht="28.5">
       <c r="F154" s="12" t="s">
         <v>17</v>
       </c>
@@ -3810,7 +5184,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="155" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="155" spans="6:13" ht="28.5">
       <c r="F155" s="12" t="s">
         <v>24</v>
       </c>
@@ -3821,7 +5195,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="156" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="156" spans="6:13" ht="28.5">
       <c r="F156" s="12" t="s">
         <v>16</v>
       </c>
@@ -3832,7 +5206,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="157" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="157" spans="6:13" ht="28.5">
       <c r="L157" s="2">
         <v>8</v>
       </c>
@@ -3840,18 +5214,18 @@
         <v>146</v>
       </c>
     </row>
-    <row r="158" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="158" spans="6:13">
       <c r="F158" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="159" spans="6:13" x14ac:dyDescent="0.45">
-      <c r="L159" s="22" t="s">
+    <row r="159" spans="6:13">
+      <c r="L159" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="M159" s="23"/>
-    </row>
-    <row r="160" spans="6:13" x14ac:dyDescent="0.45">
+      <c r="M159" s="32"/>
+    </row>
+    <row r="160" spans="6:13">
       <c r="F160" s="12" t="s">
         <v>26</v>
       </c>
@@ -3862,7 +5236,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="161" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="161" spans="6:13">
       <c r="L161" s="2">
         <v>1</v>
       </c>
@@ -3870,7 +5244,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="162" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="162" spans="6:13" ht="28.5">
       <c r="F162" s="12" t="s">
         <v>27</v>
       </c>
@@ -3881,7 +5255,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="163" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="163" spans="6:13" ht="28.5">
       <c r="L163" s="2">
         <v>3</v>
       </c>
@@ -3889,7 +5263,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="164" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="164" spans="6:13" ht="28.5">
       <c r="F164" s="12" t="s">
         <v>28</v>
       </c>
@@ -3900,16 +5274,16 @@
         <v>150</v>
       </c>
     </row>
-    <row r="166" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="166" spans="6:13">
       <c r="F166" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="L166" s="22" t="s">
+      <c r="L166" s="31" t="s">
         <v>95</v>
       </c>
-      <c r="M166" s="23"/>
-    </row>
-    <row r="167" spans="6:13" x14ac:dyDescent="0.45">
+      <c r="M166" s="32"/>
+    </row>
+    <row r="167" spans="6:13">
       <c r="L167" s="1" t="s">
         <v>125</v>
       </c>
@@ -3917,7 +5291,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="168" spans="6:13" x14ac:dyDescent="0.45">
+    <row r="168" spans="6:13">
       <c r="L168" s="2">
         <v>1</v>
       </c>
@@ -3925,7 +5299,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="169" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="169" spans="6:13" ht="28.5">
       <c r="L169" s="2">
         <v>2</v>
       </c>
@@ -3933,7 +5307,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="170" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="170" spans="6:13" ht="28.5">
       <c r="L170" s="2">
         <v>3</v>
       </c>
@@ -3941,7 +5315,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="171" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="171" spans="6:13" ht="28.5">
       <c r="L171" s="2">
         <v>4</v>
       </c>
@@ -3949,7 +5323,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="172" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="172" spans="6:13">
       <c r="L172" s="2">
         <v>5</v>
       </c>
@@ -3957,7 +5331,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="173" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="173" spans="6:13">
       <c r="L173" s="2">
         <v>6</v>
       </c>
@@ -3965,7 +5339,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="174" spans="6:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="174" spans="6:13" ht="28.5">
       <c r="L174" s="2">
         <v>7</v>
       </c>
@@ -3973,7 +5347,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="175" spans="6:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="175" spans="6:13" ht="28.5">
       <c r="L175" s="2">
         <v>8</v>
       </c>
@@ -3981,13 +5355,13 @@
         <v>157</v>
       </c>
     </row>
-    <row r="177" spans="12:13" x14ac:dyDescent="0.45">
-      <c r="L177" s="22" t="s">
+    <row r="177" spans="12:13">
+      <c r="L177" s="31" t="s">
         <v>96</v>
       </c>
-      <c r="M177" s="23"/>
-    </row>
-    <row r="178" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="M177" s="32"/>
+    </row>
+    <row r="178" spans="12:13">
       <c r="L178" s="1" t="s">
         <v>125</v>
       </c>
@@ -3995,7 +5369,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="179" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="179" spans="12:13">
       <c r="L179" s="2">
         <v>1</v>
       </c>
@@ -4003,7 +5377,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="180" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="180" spans="12:13" ht="28.5">
       <c r="L180" s="2">
         <v>2</v>
       </c>
@@ -4011,7 +5385,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="181" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="181" spans="12:13" ht="28.5">
       <c r="L181" s="2">
         <v>3</v>
       </c>
@@ -4019,7 +5393,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="182" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="182" spans="12:13" ht="28.5">
       <c r="L182" s="2">
         <v>4</v>
       </c>
@@ -4027,7 +5401,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="183" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="183" spans="12:13" ht="28.5">
       <c r="L183" s="2">
         <v>5</v>
       </c>
@@ -4035,7 +5409,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="184" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="184" spans="12:13" ht="28.5">
       <c r="L184" s="2">
         <v>6</v>
       </c>
@@ -4043,13 +5417,13 @@
         <v>163</v>
       </c>
     </row>
-    <row r="187" spans="12:13" x14ac:dyDescent="0.45">
-      <c r="L187" s="22" t="s">
+    <row r="187" spans="12:13">
+      <c r="L187" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="M187" s="23"/>
-    </row>
-    <row r="188" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="M187" s="32"/>
+    </row>
+    <row r="188" spans="12:13">
       <c r="L188" s="1" t="s">
         <v>125</v>
       </c>
@@ -4057,7 +5431,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="189" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="189" spans="12:13" ht="28.5">
       <c r="L189" s="2">
         <v>1</v>
       </c>
@@ -4065,7 +5439,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="190" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="190" spans="12:13" ht="28.5">
       <c r="L190" s="2">
         <v>2</v>
       </c>
@@ -4073,7 +5447,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="191" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="191" spans="12:13" ht="28.5">
       <c r="L191" s="2">
         <v>3</v>
       </c>
@@ -4081,7 +5455,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="192" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="192" spans="12:13" ht="28.5">
       <c r="L192" s="2">
         <v>4</v>
       </c>
@@ -4089,7 +5463,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="193" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="193" spans="12:13" ht="28.5">
       <c r="L193" s="2">
         <v>5</v>
       </c>
@@ -4097,13 +5471,13 @@
         <v>168</v>
       </c>
     </row>
-    <row r="196" spans="12:13" x14ac:dyDescent="0.45">
-      <c r="L196" s="22" t="s">
+    <row r="196" spans="12:13">
+      <c r="L196" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="M196" s="23"/>
-    </row>
-    <row r="197" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="M196" s="32"/>
+    </row>
+    <row r="197" spans="12:13">
       <c r="L197" s="1" t="s">
         <v>125</v>
       </c>
@@ -4111,7 +5485,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="198" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="198" spans="12:13">
       <c r="L198" s="2">
         <v>1</v>
       </c>
@@ -4119,7 +5493,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="199" spans="12:13" ht="28.5">
       <c r="L199" s="2">
         <v>2</v>
       </c>
@@ -4127,7 +5501,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="200" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="200" spans="12:13" ht="28.5">
       <c r="L200" s="2">
         <v>3</v>
       </c>
@@ -4135,7 +5509,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="201" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="201" spans="12:13" ht="28.5">
       <c r="L201" s="2">
         <v>4</v>
       </c>
@@ -4143,7 +5517,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="202" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="202" spans="12:13" ht="28.5">
       <c r="L202" s="2">
         <v>5</v>
       </c>
@@ -4151,7 +5525,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="203" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="203" spans="12:13" ht="28.5">
       <c r="L203" s="2">
         <v>6</v>
       </c>
@@ -4159,7 +5533,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="204" spans="12:13" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="204" spans="12:13" ht="28.5">
       <c r="L204" s="2">
         <v>7</v>
       </c>
@@ -4167,13 +5541,13 @@
         <v>174</v>
       </c>
     </row>
-    <row r="207" spans="12:13" x14ac:dyDescent="0.45">
-      <c r="L207" s="22" t="s">
+    <row r="207" spans="12:13">
+      <c r="L207" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="M207" s="23"/>
-    </row>
-    <row r="208" spans="12:13" x14ac:dyDescent="0.45">
+      <c r="M207" s="32"/>
+    </row>
+    <row r="208" spans="12:13">
       <c r="L208" s="1" t="s">
         <v>125</v>
       </c>
@@ -4181,7 +5555,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="209" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="209" spans="12:13">
       <c r="L209" s="2">
         <v>1</v>
       </c>
@@ -4189,7 +5563,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="210" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="210" spans="12:13">
       <c r="L210" s="2">
         <v>2</v>
       </c>
@@ -4197,7 +5571,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="211" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="211" spans="12:13">
       <c r="L211" s="2">
         <v>3</v>
       </c>
@@ -4205,7 +5579,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="212" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="212" spans="12:13">
       <c r="L212" s="2">
         <v>4</v>
       </c>
@@ -4213,7 +5587,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="213" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="213" spans="12:13" ht="28.5">
       <c r="L213" s="2">
         <v>5</v>
       </c>
@@ -4221,7 +5595,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="214" spans="12:13" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="214" spans="12:13" ht="28.5">
       <c r="L214" s="2">
         <v>6</v>
       </c>
@@ -4230,7 +5604,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="T3:U3"/>
     <mergeCell ref="O7:Q8"/>
     <mergeCell ref="O9:Q14"/>
@@ -4247,9 +5621,6 @@
     <mergeCell ref="L107:M107"/>
     <mergeCell ref="L97:M97"/>
     <mergeCell ref="Q20:R24"/>
-    <mergeCell ref="L74:N74"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="H17:K23"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="L5:M6"/>
@@ -4258,8 +5629,1527 @@
     <mergeCell ref="H9:J14"/>
     <mergeCell ref="H7:J8"/>
     <mergeCell ref="Q79:R79"/>
+    <mergeCell ref="L29:O29"/>
+    <mergeCell ref="L74:N74"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="H17:K23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5005759E-BA52-4AB7-B528-2C2941D382FE}">
+  <dimension ref="B2:B407"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="116.19921875" style="36" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" ht="30.75">
+      <c r="B2" s="35" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2">
+      <c r="B3" s="36" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" s="16" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2">
+      <c r="B6" s="16" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" s="16" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" s="16" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" s="16" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2">
+      <c r="B10" s="16" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2">
+      <c r="B12" s="36" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" s="37"/>
+    </row>
+    <row r="14" spans="2:2">
+      <c r="B14" s="37" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" s="37" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2">
+      <c r="B16" s="37" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="37" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" s="37" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="37" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="37" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="37" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" s="36" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" ht="30.75">
+      <c r="B26" s="35" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="7"/>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" s="16" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="16" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" s="16" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2">
+      <c r="B32" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" s="16" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" ht="17.649999999999999">
+      <c r="B39" s="38" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2">
+      <c r="B40" s="37"/>
+    </row>
+    <row r="41" spans="2:2">
+      <c r="B41" s="39" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2">
+      <c r="B42" s="39" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2">
+      <c r="B43" s="39" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" ht="28.5">
+      <c r="B44" s="39" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" ht="30.75">
+      <c r="B48" s="35" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2">
+      <c r="B49" s="7"/>
+    </row>
+    <row r="50" spans="2:2">
+      <c r="B50" s="16" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2">
+      <c r="B51" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2">
+      <c r="B52" s="16" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2">
+      <c r="B53" s="16" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2">
+      <c r="B54" s="16" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2">
+      <c r="B55" s="16" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" ht="23.25">
+      <c r="B57" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" ht="28.5">
+      <c r="B59" s="41" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" ht="28.5">
+      <c r="B61" s="41" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" ht="23.25">
+      <c r="B63" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2">
+      <c r="B64" s="37"/>
+    </row>
+    <row r="65" spans="2:2">
+      <c r="B65" s="37" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2">
+      <c r="B66" s="37" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2">
+      <c r="B67" s="37" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2">
+      <c r="B68" s="37" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2">
+      <c r="B69" s="37" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2">
+      <c r="B70" s="37" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2">
+      <c r="B71" s="37" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" ht="30.75">
+      <c r="B73" s="35" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2">
+      <c r="B74" s="7"/>
+    </row>
+    <row r="75" spans="2:2">
+      <c r="B75" s="16" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2">
+      <c r="B76" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2">
+      <c r="B77" s="16" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2">
+      <c r="B78" s="16" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2">
+      <c r="B79" s="16" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2">
+      <c r="B80" s="16" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" ht="23.25">
+      <c r="B82" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="84" spans="2:2" ht="28.5">
+      <c r="B84" s="41" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" ht="28.5">
+      <c r="B85" s="41" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" ht="23.25">
+      <c r="B87" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2">
+      <c r="B88" s="37"/>
+    </row>
+    <row r="89" spans="2:2">
+      <c r="B89" s="37" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2">
+      <c r="B90" s="37" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2">
+      <c r="B91" s="37" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2">
+      <c r="B92" s="37" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2">
+      <c r="B93" s="37" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2">
+      <c r="B94" s="37" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2">
+      <c r="B95" s="37" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="98" spans="2:2" ht="30.75">
+      <c r="B98" s="35" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="99" spans="2:2">
+      <c r="B99" s="7"/>
+    </row>
+    <row r="100" spans="2:2">
+      <c r="B100" s="16" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="101" spans="2:2">
+      <c r="B101" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="102" spans="2:2">
+      <c r="B102" s="16" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="103" spans="2:2">
+      <c r="B103" s="16" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="104" spans="2:2">
+      <c r="B104" s="16" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="105" spans="2:2">
+      <c r="B105" s="16" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="106" spans="2:2">
+      <c r="B106" s="16" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="107" spans="2:2">
+      <c r="B107" s="16" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="109" spans="2:2" ht="30.75">
+      <c r="B109" s="35" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="110" spans="2:2" ht="17.649999999999999">
+      <c r="B110" s="38" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="111" spans="2:2">
+      <c r="B111" s="36" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="112" spans="2:2" ht="17.649999999999999">
+      <c r="B112" s="38" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2">
+      <c r="B113" s="36" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2" ht="17.649999999999999">
+      <c r="B114" s="38" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2">
+      <c r="B115" s="36" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="116" spans="2:2" ht="17.649999999999999">
+      <c r="B116" s="38" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="117" spans="2:2">
+      <c r="B117" s="36" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" ht="17.649999999999999">
+      <c r="B118" s="38" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="119" spans="2:2">
+      <c r="B119" s="36" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="120" spans="2:2" ht="17.649999999999999">
+      <c r="B120" s="38" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2">
+      <c r="B121" s="36" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="123" spans="2:2" ht="30.75">
+      <c r="B123" s="35" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="124" spans="2:2">
+      <c r="B124" s="37"/>
+    </row>
+    <row r="125" spans="2:2">
+      <c r="B125" s="37" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="126" spans="2:2">
+      <c r="B126" s="37" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="127" spans="2:2">
+      <c r="B127" s="37" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="128" spans="2:2">
+      <c r="B128" s="37" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2">
+      <c r="B129" s="37" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="130" spans="2:2">
+      <c r="B130" s="37" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="131" spans="2:2">
+      <c r="B131" s="37" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="134" spans="2:2" ht="30.75">
+      <c r="B134" s="35" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="135" spans="2:2">
+      <c r="B135" s="7"/>
+    </row>
+    <row r="136" spans="2:2">
+      <c r="B136" s="16" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2">
+      <c r="B137" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2">
+      <c r="B138" s="16" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="139" spans="2:2">
+      <c r="B139" s="16" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="140" spans="2:2">
+      <c r="B140" s="16" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="141" spans="2:2">
+      <c r="B141" s="16" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="142" spans="2:2">
+      <c r="B142" s="16" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="143" spans="2:2">
+      <c r="B143" s="16" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="144" spans="2:2">
+      <c r="B144" s="16" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="145" spans="2:2">
+      <c r="B145" s="16" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="146" spans="2:2">
+      <c r="B146" s="16" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="147" spans="2:2">
+      <c r="B147" s="16" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="151" spans="2:2" ht="30.75">
+      <c r="B151" s="35" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="153" spans="2:2">
+      <c r="B153" s="41" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="154" spans="2:2">
+      <c r="B154" s="36" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="156" spans="2:2">
+      <c r="B156" s="41" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="157" spans="2:2">
+      <c r="B157" s="36" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="159" spans="2:2">
+      <c r="B159" s="41" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="160" spans="2:2">
+      <c r="B160" s="36" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="162" spans="2:2">
+      <c r="B162" s="41" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="163" spans="2:2">
+      <c r="B163" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="165" spans="2:2">
+      <c r="B165" s="41" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="166" spans="2:2">
+      <c r="B166" s="36" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="170" spans="2:2" ht="30.75">
+      <c r="B170" s="35" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="171" spans="2:2">
+      <c r="B171" s="37"/>
+    </row>
+    <row r="172" spans="2:2">
+      <c r="B172" s="37" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="173" spans="2:2">
+      <c r="B173" s="37" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="174" spans="2:2">
+      <c r="B174" s="37" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="175" spans="2:2">
+      <c r="B175" s="37" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="176" spans="2:2">
+      <c r="B176" s="37" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="177" spans="2:2">
+      <c r="B177" s="37" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="178" spans="2:2">
+      <c r="B178" s="37" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="179" spans="2:2">
+      <c r="B179" s="37" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="180" spans="2:2">
+      <c r="B180" s="37" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="183" spans="2:2" ht="30.75">
+      <c r="B183" s="35" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="184" spans="2:2">
+      <c r="B184" s="7"/>
+    </row>
+    <row r="185" spans="2:2">
+      <c r="B185" s="16" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="186" spans="2:2">
+      <c r="B186" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="187" spans="2:2">
+      <c r="B187" s="16" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="188" spans="2:2">
+      <c r="B188" s="16" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="189" spans="2:2">
+      <c r="B189" s="16" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="190" spans="2:2">
+      <c r="B190" s="16" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="192" spans="2:2" ht="23.25">
+      <c r="B192" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="194" spans="2:2">
+      <c r="B194" s="41" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="195" spans="2:2">
+      <c r="B195" s="36" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="197" spans="2:2">
+      <c r="B197" s="41" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="198" spans="2:2" ht="28.5">
+      <c r="B198" s="36" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="202" spans="2:2" ht="23.25">
+      <c r="B202" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="203" spans="2:2">
+      <c r="B203" s="37"/>
+    </row>
+    <row r="204" spans="2:2">
+      <c r="B204" s="37" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="205" spans="2:2">
+      <c r="B205" s="37" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="206" spans="2:2">
+      <c r="B206" s="37" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="207" spans="2:2">
+      <c r="B207" s="37" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="208" spans="2:2">
+      <c r="B208" s="37" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="209" spans="2:2">
+      <c r="B209" s="37" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="210" spans="2:2">
+      <c r="B210" s="37" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="211" spans="2:2">
+      <c r="B211" s="37" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="215" spans="2:2" ht="30.75">
+      <c r="B215" s="35" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="216" spans="2:2">
+      <c r="B216" s="7"/>
+    </row>
+    <row r="217" spans="2:2">
+      <c r="B217" s="16" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="218" spans="2:2">
+      <c r="B218" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="219" spans="2:2">
+      <c r="B219" s="16" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="220" spans="2:2">
+      <c r="B220" s="16" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="221" spans="2:2">
+      <c r="B221" s="16" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="222" spans="2:2">
+      <c r="B222" s="16" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="224" spans="2:2" ht="23.25">
+      <c r="B224" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="226" spans="2:2">
+      <c r="B226" s="41" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="227" spans="2:2" ht="28.5">
+      <c r="B227" s="36" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="229" spans="2:2">
+      <c r="B229" s="41" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="230" spans="2:2" ht="28.5">
+      <c r="B230" s="36" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="234" spans="2:2" ht="23.25">
+      <c r="B234" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="235" spans="2:2">
+      <c r="B235" s="37"/>
+    </row>
+    <row r="236" spans="2:2">
+      <c r="B236" s="37" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="237" spans="2:2">
+      <c r="B237" s="37" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="238" spans="2:2">
+      <c r="B238" s="37" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="239" spans="2:2">
+      <c r="B239" s="37" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="240" spans="2:2">
+      <c r="B240" s="37" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="241" spans="2:2">
+      <c r="B241" s="37" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="242" spans="2:2">
+      <c r="B242" s="37" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="243" spans="2:2">
+      <c r="B243" s="37" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="244" spans="2:2">
+      <c r="B244" s="37" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="245" spans="2:2">
+      <c r="B245" s="37" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="248" spans="2:2" ht="30.75">
+      <c r="B248" s="35" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="249" spans="2:2">
+      <c r="B249" s="7"/>
+    </row>
+    <row r="250" spans="2:2">
+      <c r="B250" s="16" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="251" spans="2:2">
+      <c r="B251" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="252" spans="2:2">
+      <c r="B252" s="16" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="253" spans="2:2">
+      <c r="B253" s="16" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="254" spans="2:2">
+      <c r="B254" s="16" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="255" spans="2:2">
+      <c r="B255" s="16" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="256" spans="2:2">
+      <c r="B256" s="16" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="257" spans="2:2">
+      <c r="B257" s="16" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="259" spans="2:2" ht="23.25">
+      <c r="B259" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="261" spans="2:2">
+      <c r="B261" s="41" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="262" spans="2:2" ht="28.5">
+      <c r="B262" s="36" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="264" spans="2:2">
+      <c r="B264" s="41" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="265" spans="2:2" ht="28.5">
+      <c r="B265" s="36" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="267" spans="2:2">
+      <c r="B267" s="41" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="268" spans="2:2">
+      <c r="B268" s="36" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="272" spans="2:2" ht="23.25">
+      <c r="B272" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="273" spans="2:2">
+      <c r="B273" s="37"/>
+    </row>
+    <row r="274" spans="2:2">
+      <c r="B274" s="37" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="275" spans="2:2">
+      <c r="B275" s="37" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="276" spans="2:2">
+      <c r="B276" s="37" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="277" spans="2:2">
+      <c r="B277" s="37" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="278" spans="2:2">
+      <c r="B278" s="37" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="279" spans="2:2">
+      <c r="B279" s="37" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="280" spans="2:2">
+      <c r="B280" s="37" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="281" spans="2:2">
+      <c r="B281" s="37" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="284" spans="2:2" ht="30.75">
+      <c r="B284" s="35" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="285" spans="2:2">
+      <c r="B285" s="7"/>
+    </row>
+    <row r="286" spans="2:2">
+      <c r="B286" s="16" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="287" spans="2:2">
+      <c r="B287" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="288" spans="2:2">
+      <c r="B288" s="16" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="289" spans="2:2">
+      <c r="B289" s="16" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="291" spans="2:2" ht="23.25">
+      <c r="B291" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="293" spans="2:2">
+      <c r="B293" s="41" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="294" spans="2:2" ht="28.5">
+      <c r="B294" s="36" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="298" spans="2:2" ht="23.25">
+      <c r="B298" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="299" spans="2:2">
+      <c r="B299" s="37"/>
+    </row>
+    <row r="300" spans="2:2">
+      <c r="B300" s="37" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="301" spans="2:2">
+      <c r="B301" s="37" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="302" spans="2:2">
+      <c r="B302" s="37" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="303" spans="2:2">
+      <c r="B303" s="37" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="304" spans="2:2">
+      <c r="B304" s="37" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="305" spans="2:2">
+      <c r="B305" s="37" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="308" spans="2:2" ht="30.75">
+      <c r="B308" s="35" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="309" spans="2:2">
+      <c r="B309" s="7"/>
+    </row>
+    <row r="310" spans="2:2">
+      <c r="B310" s="16" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="311" spans="2:2">
+      <c r="B311" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="312" spans="2:2">
+      <c r="B312" s="16" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="313" spans="2:2">
+      <c r="B313" s="16" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="315" spans="2:2" ht="23.25">
+      <c r="B315" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="317" spans="2:2">
+      <c r="B317" s="41" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="318" spans="2:2" ht="28.5">
+      <c r="B318" s="36" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="322" spans="2:2" ht="23.25">
+      <c r="B322" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="323" spans="2:2">
+      <c r="B323" s="37"/>
+    </row>
+    <row r="324" spans="2:2">
+      <c r="B324" s="37" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="325" spans="2:2">
+      <c r="B325" s="37" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="326" spans="2:2">
+      <c r="B326" s="37" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="327" spans="2:2">
+      <c r="B327" s="37" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="328" spans="2:2">
+      <c r="B328" s="37" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="329" spans="2:2">
+      <c r="B329" s="37" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="330" spans="2:2">
+      <c r="B330" s="37" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="333" spans="2:2" ht="30.75">
+      <c r="B333" s="35" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="334" spans="2:2">
+      <c r="B334" s="7"/>
+    </row>
+    <row r="335" spans="2:2">
+      <c r="B335" s="16" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="336" spans="2:2">
+      <c r="B336" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="337" spans="2:2">
+      <c r="B337" s="16" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="338" spans="2:2">
+      <c r="B338" s="16" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="340" spans="2:2" ht="23.25">
+      <c r="B340" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="342" spans="2:2">
+      <c r="B342" s="41" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="343" spans="2:2" ht="28.5">
+      <c r="B343" s="36" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="347" spans="2:2" ht="23.25">
+      <c r="B347" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="348" spans="2:2">
+      <c r="B348" s="37"/>
+    </row>
+    <row r="349" spans="2:2">
+      <c r="B349" s="37" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="350" spans="2:2">
+      <c r="B350" s="37" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="351" spans="2:2">
+      <c r="B351" s="37" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="352" spans="2:2">
+      <c r="B352" s="37" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="353" spans="2:2">
+      <c r="B353" s="37" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="354" spans="2:2">
+      <c r="B354" s="37" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="355" spans="2:2">
+      <c r="B355" s="37" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="358" spans="2:2" ht="30.75">
+      <c r="B358" s="35" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="359" spans="2:2">
+      <c r="B359" s="7"/>
+    </row>
+    <row r="360" spans="2:2">
+      <c r="B360" s="16" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="361" spans="2:2">
+      <c r="B361" s="16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="362" spans="2:2">
+      <c r="B362" s="16" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="363" spans="2:2">
+      <c r="B363" s="16" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="364" spans="2:2">
+      <c r="B364" s="16" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="366" spans="2:2" ht="23.25">
+      <c r="B366" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="368" spans="2:2">
+      <c r="B368" s="41" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="369" spans="2:2" ht="28.5">
+      <c r="B369" s="36" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="371" spans="2:2">
+      <c r="B371" s="41" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="372" spans="2:2">
+      <c r="B372" s="36" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="376" spans="2:2" ht="23.25">
+      <c r="B376" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="377" spans="2:2">
+      <c r="B377" s="37"/>
+    </row>
+    <row r="378" spans="2:2">
+      <c r="B378" s="37" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="379" spans="2:2">
+      <c r="B379" s="37" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="380" spans="2:2">
+      <c r="B380" s="37" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="381" spans="2:2">
+      <c r="B381" s="37" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="382" spans="2:2">
+      <c r="B382" s="37" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="385" spans="2:2" ht="30.75">
+      <c r="B385" s="35" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="386" spans="2:2">
+      <c r="B386" s="7"/>
+    </row>
+    <row r="387" spans="2:2">
+      <c r="B387" s="16" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="388" spans="2:2">
+      <c r="B388" s="16" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="389" spans="2:2">
+      <c r="B389" s="16" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="390" spans="2:2">
+      <c r="B390" s="16" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="392" spans="2:2" ht="23.25">
+      <c r="B392" s="40" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="394" spans="2:2">
+      <c r="B394" s="41" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="395" spans="2:2" ht="42.75">
+      <c r="B395" s="36" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="399" spans="2:2" ht="23.25">
+      <c r="B399" s="40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="400" spans="2:2">
+      <c r="B400" s="37"/>
+    </row>
+    <row r="401" spans="2:2">
+      <c r="B401" s="37" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="402" spans="2:2">
+      <c r="B402" s="37" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="403" spans="2:2">
+      <c r="B403" s="37" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="404" spans="2:2">
+      <c r="B404" s="37" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="405" spans="2:2">
+      <c r="B405" s="37" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="406" spans="2:2">
+      <c r="B406" s="37" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="407" spans="2:2">
+      <c r="B407" s="37" t="s">
+        <v>596</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>